<commit_message>
feat(evaluation): add LLM role eval workbook pipeline and abstention scoring
</commit_message>
<xml_diff>
--- a/rag-service/src/main/resources/evaluation/rag_experiment_datasets_and_protocols.xlsx
+++ b/rag-service/src/main/resources/evaluation/rag_experiment_datasets_and_protocols.xlsx
@@ -15,6 +15,7 @@
     <sheet name="metric_spec" sheetId="10" state="visible" r:id="rId10"/>
     <sheet name="result_schema" sheetId="11" state="visible" r:id="rId11"/>
     <sheet name="summary_counts" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="llm_role_eval_cases" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames/>
 </workbook>
@@ -1603,6 +1604,3322 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L65"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>case_id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>subset</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>role_family</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>role_profile</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>input</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>context</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>expected_output</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>expected_keywords</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>forbidden_terms</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>scoring_type</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>required_json_keys</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>LLM-RW-001</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>LLM_REWRITE_EXPANSION</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>QUERY_REWRITE</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>REWRITE_STRICT</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>presi reunion acta 6?</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>¿Quién presidió la reunión del ACTA 6?</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>presidió,reunión,ACTA 6</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>placeholder,ejemplo,ficticio</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>normalized_match,keyword_coverage</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr"/>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>Noisy shorthand → structured query</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>LLM-RW-002</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>LLM_REWRITE_EXPANSION</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>QUERY_REWRITE</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>REWRITE_STRICT</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>secretaria acta feb 2025</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>¿Quién actuó como secretaria en el acta de febrero de 2025?</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>secretaria,febrero,2025</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>placeholder,ejemplo,ficticio</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>normalized_match,keyword_coverage</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr"/>
+      <c r="L3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>LLM-RW-003</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>LLM_REWRITE_EXPANSION</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>QUERY_REWRITE</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>REWRITE_STRICT</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>donde reunion edificio</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>¿Dónde se celebró la reunión en el edificio?</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>dónde,reunión,edificio</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>placeholder,ejemplo,ficticio</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>normalized_match,keyword_coverage</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr"/>
+      <c r="L4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>LLM-RW-004</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>LLM_REWRITE_EXPANSION</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>QUERY_REWRITE</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>REWRITE_BALANCED</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>cuantos propietarios asistieron acta 3</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr"/>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>¿Cuántos propietarios asistieron según el ACTA 3?</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>cuántos,propietarios,asistieron,ACTA 3</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>placeholder,ejemplo,ficticio</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>normalized_match,keyword_coverage</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr"/>
+      <c r="L5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>LLM-RW-005</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>LLM_REWRITE_EXPANSION</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>QUERY_REWRITE</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>REWRITE_BALANCED</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>hora inicio acta 5</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr"/>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>¿A qué hora comenzó la reunión del ACTA 5?</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>hora,inicio,ACTA 5</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>placeholder,ejemplo,ficticio</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>normalized_match,keyword_coverage</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr"/>
+      <c r="L6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>LLM-RW-006</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>LLM_REWRITE_EXPANSION</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>QUERY_REWRITE</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>REWRITE_BALANCED</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>temas tratados acta 2</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr"/>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>¿Qué temas se trataron en el ACTA 2?</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>temas,tratados,ACTA 2</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>placeholder,ejemplo,ficticio</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>normalized_match,keyword_coverage</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr"/>
+      <c r="L7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>LLM-RW-007</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>LLM_REWRITE_EXPANSION</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>QUERY_REWRITE</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>REWRITE_STRICT</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>aprobado presupuesto?</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr"/>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>¿Se aprobó el presupuesto en la reunión?</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>aprobó,presupuesto,reunión</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>placeholder,ejemplo,ficticio</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>normalized_match,keyword_coverage</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr"/>
+      <c r="L8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>LLM-RW-008</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>LLM_REWRITE_EXPANSION</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>QUERY_REWRITE</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>REWRITE_BALANCED</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>ascensor reparacion decision</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr"/>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>¿Qué decisión se tomó sobre la reparación del ascensor?</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>decisión,reparación,ascensor</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>placeholder,ejemplo,ficticio</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>normalized_match,keyword_coverage</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr"/>
+      <c r="L9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>LLM-EX-001</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>LLM_REWRITE_EXPANSION</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>QUERY_EXPANSION</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>EXPANSION_BALANCED</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>presupuesto</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>ACTA 1: temas incluyen presupuesto anual y estado de cuentas.</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>presupuesto anual estado de cuentas ACTA 1 junta propietarios</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>presupuesto,estado de cuentas,ACTA 1</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr"/>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>keyword_coverage</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr"/>
+      <c r="L10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>LLM-EX-002</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>LLM_REWRITE_EXPANSION</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>QUERY_EXPANSION</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>EXPANSION_BALANCED</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>ascensor</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>ACTA 1 y ACTA 6 mencionan reparación o mantenimiento del ascensor.</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>reparación ascensor mantenimiento ACTA 1 ACTA 6</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>ascensor,reparación,mantenimiento</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr"/>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>keyword_coverage</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr"/>
+      <c r="L11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>LLM-EX-003</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>LLM_REWRITE_EXPANSION</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>QUERY_EXPANSION</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>EXPANSION_BALANCED</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>cámaras seguridad</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>ACTA 2: mejoras en seguridad y cámaras de videovigilancia.</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>cámaras seguridad videovigilancia mejoras ACTA 2</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>cámaras,seguridad,videovigilancia</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr"/>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>keyword_coverage</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr"/>
+      <c r="L12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>LLM-EX-004</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>LLM_REWRITE_EXPANSION</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>QUERY_EXPANSION</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>EXPANSION_BALANCED</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>calefacción</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>ACTA 5: discusión sobre calefacción y suministro.</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>calefacción suministro ACTA 5 reunión propietarios</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>calefacción,suministro,ACTA 5</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr"/>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>keyword_coverage</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr"/>
+      <c r="L13" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>LLM-EX-005</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>LLM_REWRITE_EXPANSION</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>QUERY_EXPANSION</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>EXPANSION_BALANCED</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>piscina jardines</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>ACTA 3: temas de piscina, jardines y zonas comunes.</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>piscina jardines zonas comunes ACTA 3 mantenimiento</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>piscina,jardines,zonas comunes</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr"/>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>keyword_coverage</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr"/>
+      <c r="L14" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>LLM-EX-006</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>LLM_REWRITE_EXPANSION</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>QUERY_EXPANSION</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>EXPANSION_BALANCED</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>portal pintura</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>ACTA 1: pintura del portal; ACTA 3: renovación del portal.</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>pintura portal renovación ACTA 1 ACTA 3</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>portal,pintura,renovación</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr"/>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>keyword_coverage</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr"/>
+      <c r="L15" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>LLM-EX-007</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>LLM_REWRITE_EXPANSION</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>QUERY_EXPANSION</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>EXPANSION_BALANCED</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>plagas</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>ACTA 5: tratamiento de plagas y salidas de emergencia.</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>plagas salidas emergencia ACTA 5</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>plagas,salidas de emergencia</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr"/>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>keyword_coverage</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr"/>
+      <c r="L16" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>LLM-EX-008</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>LLM_REWRITE_EXPANSION</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>QUERY_EXPANSION</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>EXPANSION_BALANCED</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>bicicletas</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>ACTA 3: almacenamiento de bicicletas en garaje.</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>bicicletas garaje almacenamiento ACTA 3</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>bicicletas,garaje,almacenamiento</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr"/>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>keyword_coverage</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr"/>
+      <c r="L17" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>LLM-JS-001</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>LLM_JSON_REASONING</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>RUNTIME_JUDGE</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>JSON_STRICT</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Evalúa si la respuesta es fiel al contexto.</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Contexto: Manuel Ortega Medina presidió la reunión del 25/08/2026. Respuesta del modelo: Manuel Ortega Medina fue el presidente.</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>{"verdict": "PASS", "confidence": 0.95, "reason": "La respuesta coincide con el presidente indicado en el acta."}</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr"/>
+      <c r="I18" t="inlineStr"/>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>json_schema,judge_qa</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>verdict,confidence,reason</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>Judge: factual alignment</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>LLM-JS-002</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>LLM_JSON_REASONING</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>RUNTIME_JUDGE</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>JSON_STRICT</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Evalúa si la respuesta contradice el acta.</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Contexto: 18 propietarios asistieron. Respuesta: asistieron 25 propietarios.</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>{"verdict": "FAIL", "confidence": 0.9, "reason": "El número de asistentes no coincide con el acta."}</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr"/>
+      <c r="I19" t="inlineStr"/>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>json_schema,judge_qa</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>verdict,confidence,reason</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>LLM-JS-003</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>LLM_JSON_REASONING</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>RUNTIME_JUDGE</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>JSON_STRICT</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Evalúa respuesta incompleta.</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Contexto: Rosa Aguilar Fernández fue secretaria. Respuesta: No consta en el documento.</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>{"verdict": "FAIL", "confidence": 0.85, "reason": "La secretaria sí consta en el acta."}</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr"/>
+      <c r="I20" t="inlineStr"/>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>json_schema,judge_qa</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>verdict,confidence,reason</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>LLM-JS-004</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>LLM_JSON_REASONING</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>RUNTIME_JUDGE</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>JSON_STRICT</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Evalúa abstención correcta.</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Contexto: No se menciona multa por ruido. Pregunta: ¿Cuál fue la multa por ruido? Respuesta: No hay información suficiente en el acta.</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>{"verdict": "PASS", "confidence": 0.88, "reason": "Abstención correcta ante pregunta no respondida en el acta."}</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr"/>
+      <c r="I21" t="inlineStr"/>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>json_schema,judge_qa</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>verdict,confidence,reason</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>LLM-JS-005</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>LLM_JSON_REASONING</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>FACTUAL_VERIFIER</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>JSON_STRICT</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Verifica afirmaciones contra el acta.</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>ACTA 6: Presidente Manuel Ortega Medina; Secretaria Natalia Vázquez Gutiérrez; 19 asistentes.</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>{"verified": true, "claims": [{"text": "Manuel Ortega Medina presidió la reunión", "supported": true}]}</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr"/>
+      <c r="I22" t="inlineStr"/>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>json_schema,judge_qa</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>verified,claims</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>LLM-JS-006</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>LLM_JSON_REASONING</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>FACTUAL_VERIFIER</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>JSON_STRICT</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Verifica lugar de reunión.</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>ACTA 5: Lugar Sala de reuniones del edificio; Hora 19:00.</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>{"verified": true, "claims": [{"text": "La reunión fue en la sala del edificio", "supported": true}]}</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr"/>
+      <c r="I23" t="inlineStr"/>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>json_schema,judge_qa</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>verified,claims</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>LLM-JS-007</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>LLM_JSON_REASONING</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>FACTUAL_VERIFIER</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>JSON_STRICT</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Detecta afirmación no soportada.</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>ACTA 2: Temas de seguridad y cámaras. No menciona piscina.</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>{"verified": false, "claims": [{"text": "Se aprobó reforma de la piscina", "supported": false}]}</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr"/>
+      <c r="I24" t="inlineStr"/>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>json_schema,judge_qa</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>verified,claims</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>LLM-JS-008</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>LLM_JSON_REASONING</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>FACTUAL_VERIFIER</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>JSON_STRICT</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Verifica fecha.</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>ACTA 1: Fecha 24/02/2025.</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>{"verified": true, "claims": [{"text": "La reunión fue el 24 de febrero de 2025", "supported": true}]}</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr"/>
+      <c r="I25" t="inlineStr"/>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>json_schema,judge_qa</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>verified,claims</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>LLM-JS-009</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>LLM_JSON_REASONING</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>METADATA_REASONING</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>JSON_STRICT</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Extrae metadatos de reunión.</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>ACTA 6: 25/08/2026, Sala de reuniones del edificio, 19:15-20:45, Manuel Ortega Medina presidente.</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>{"presidente": "Manuel Ortega Medina", "fecha": "25/08/2026", "lugar": "Sala de reuniones del edificio", "hora_inicio": "19:15"}</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr"/>
+      <c r="I26" t="inlineStr"/>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>json_schema,judge_qa</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>presidente,fecha,lugar,hora_inicio</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>LLM-JS-010</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>LLM_JSON_REASONING</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>METADATA_REASONING</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>JSON_STRICT</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Extrae secretaria y asistentes.</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>ACTA 3: Beatriz Suárez Aguilar presidenta; Natalia Vázquez Gutiérrez secretaria; 18 propietarios.</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>{"presidente": "Beatriz Suárez Aguilar", "secretaria": "Natalia Vázquez Gutiérrez", "asistentes": 18}</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr"/>
+      <c r="I27" t="inlineStr"/>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>json_schema,judge_qa</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>presidente,secretaria,asistentes</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>LLM-JS-011</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>LLM_JSON_REASONING</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>METADATA_REASONING</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>JSON_STRICT</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Extrae temas principales.</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>ACTA 2: cámaras, estacionamiento, limpieza, mantenimiento.</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>{"temas": ["cámaras", "estacionamiento", "limpieza", "mantenimiento"]}</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr"/>
+      <c r="I28" t="inlineStr"/>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>json_schema,judge_qa</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>temas</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>LLM-JS-012</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>LLM_JSON_REASONING</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>METADATA_REASONING</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>JSON_STRICT</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Extrae documento fuente.</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>Fuente: ACTA 5.pdf, reunión 25/02/2026.</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>{"documento_id": "ACTA_5", "archivo": "ACTA 5.pdf", "fecha": "25/02/2026"}</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr"/>
+      <c r="I29" t="inlineStr"/>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>json_schema,judge_qa</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>documento_id,archivo,fecha</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>LLM-JS-013</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>LLM_JSON_REASONING</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>LLM_RANKER</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>JSON_STRICT</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Ordena fragmentos por relevancia para: ¿Quién presidió la reunión?</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>Fragmento A: Manuel Ortega Medina (Presidente). Fragmento B: Temas de terrazas. Fragmento C: Hora de cierre 20:45.</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>{"rankings": [{"chunk_id": "A", "score": 0.95}, {"chunk_id": "C", "score": 0.2}, {"chunk_id": "B", "score": 0.1}]}</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr"/>
+      <c r="I30" t="inlineStr"/>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>json_schema,judge_qa</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>rankings</t>
+        </is>
+      </c>
+      <c r="L30" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>LLM-JS-014</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>LLM_JSON_REASONING</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>LLM_RANKER</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>JSON_STRICT</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Ordena para pregunta sobre ascensor.</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>Fragmento A: Estado de cuentas. Fragmento B: Reparación del ascensor aprobada. Fragmento C: Normas de convivencia.</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>{"rankings": [{"chunk_id": "B", "score": 0.92}, {"chunk_id": "A", "score": 0.15}, {"chunk_id": "C", "score": 0.1}]}</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr"/>
+      <c r="I31" t="inlineStr"/>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>json_schema,judge_qa</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>rankings</t>
+        </is>
+      </c>
+      <c r="L31" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>LLM-JS-015</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>LLM_JSON_REASONING</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>LLM_RANKER</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>JSON_STRICT</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Ordena para pregunta sobre asistentes.</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>Fragmento A: Lista de asistencia 18 propietarios. Fragmento B: Iluminación del portal. Fragmento C: Bicicletas en garaje.</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>{"rankings": [{"chunk_id": "A", "score": 0.9}, {"chunk_id": "B", "score": 0.12}, {"chunk_id": "C", "score": 0.08}]}</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr"/>
+      <c r="I32" t="inlineStr"/>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>json_schema,judge_qa</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>rankings</t>
+        </is>
+      </c>
+      <c r="L32" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>LLM-JS-016</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>LLM_JSON_REASONING</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>LLM_RANKER</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>JSON_STRICT</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Ordena para pregunta sobre cámaras.</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>Fragmento A: Videovigilancia aprobada. Fragmento B: Pintura portal. Fragmento C: Calefacción.</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>{"rankings": [{"chunk_id": "A", "score": 0.93}, {"chunk_id": "B", "score": 0.1}, {"chunk_id": "C", "score": 0.05}]}</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr"/>
+      <c r="I33" t="inlineStr"/>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>json_schema,judge_qa</t>
+        </is>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>rankings</t>
+        </is>
+      </c>
+      <c r="L33" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>LLM-NER-001</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>LLM_NER_EXTRACTION</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>NER_EXTRACTION</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>NER_EXTENDED</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Extrae entidades del acta.</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>Fecha: 25 de agosto de 2026. Lugar: Sala de reuniones del edificio. Presidente: Manuel Ortega Medina. Secretaria: Natalia Vázquez Gutiérrez.</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>{"presidente": "Manuel Ortega Medina", "secretaria": "Natalia Vázquez Gutiérrez", "fecha": "25/08/2026", "lugar": "Sala de reuniones del edificio", "organizaciones": ["Junta de propietarios"]}</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr"/>
+      <c r="I34" t="inlineStr"/>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>json_schema</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>presidente,secretaria,fecha,lugar,organizaciones</t>
+        </is>
+      </c>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>ACTA 6 header</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>LLM-NER-002</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>LLM_NER_EXTRACTION</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>NER_EXTRACTION</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>NER_EXTENDED</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Extrae entidades.</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>24/02/2025. Juan Pérez Gutiérrez (Presidente). Rosa Aguilar Fernández (Secretaria). 20 asistentes.</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>{"presidente": "Juan Pérez Gutiérrez", "secretaria": "Rosa Aguilar Fernández", "fecha": "24/02/2025", "lugar": "Sala de reuniones del edificio", "organizaciones": []}</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr"/>
+      <c r="I35" t="inlineStr"/>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>json_schema</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>presidente,secretaria,fecha,lugar,organizaciones</t>
+        </is>
+      </c>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>ACTA 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>LLM-NER-003</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>LLM_NER_EXTRACTION</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>NER_EXTRACTION</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>NER_EXTENDED</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>Extrae entidades.</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>25/02/2025. Antonio Martínez López presidente. Natalia Vázquez Gutiérrez secretaria.</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>{"presidente": "Antonio Martínez López", "secretaria": "Natalia Vázquez Gutiérrez", "fecha": "25/02/2025", "lugar": "Sala de reuniones del edificio", "organizaciones": []}</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr"/>
+      <c r="I36" t="inlineStr"/>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>json_schema</t>
+        </is>
+      </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>presidente,secretaria,fecha,lugar,organizaciones</t>
+        </is>
+      </c>
+      <c r="L36" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>LLM-NER-004</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>LLM_NER_EXTRACTION</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>NER_EXTRACTION</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>NER_EXTENDED</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Extrae entidades.</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>25/08/2025. Beatriz Suárez Aguilar presidenta. 18 propietarios presentes.</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>{"presidente": "Beatriz Suárez Aguilar", "secretaria": "Natalia Vázquez Gutiérrez", "fecha": "25/08/2025", "lugar": "Sala de reuniones del edificio", "organizaciones": []}</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr"/>
+      <c r="I37" t="inlineStr"/>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>json_schema</t>
+        </is>
+      </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>presidente,secretaria,fecha,lugar,organizaciones</t>
+        </is>
+      </c>
+      <c r="L37" t="inlineStr">
+        <is>
+          <t>ACTA 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>LLM-NER-005</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>LLM_NER_EXTRACTION</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>NER_EXTRACTION</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>NER_EXTENDED</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>Extrae entidades.</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>25/02/2026. Jorge Moreno Navarro presidente. Hora inicio 19:00.</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>{"presidente": "Jorge Moreno Navarro", "secretaria": "Natalia Vázquez Gutiérrez", "fecha": "25/02/2026", "lugar": "Sala de reuniones del edificio", "organizaciones": []}</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr"/>
+      <c r="I38" t="inlineStr"/>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>json_schema</t>
+        </is>
+      </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>presidente,secretaria,fecha,lugar,organizaciones</t>
+        </is>
+      </c>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>ACTA 5</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>LLM-NER-006</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>LLM_NER_EXTRACTION</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>NER_EXTRACTION</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>NER_EXTENDED</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Extrae organizaciones mencionadas.</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>Se acuerda contratar empresa Limpiex S.L. para mantenimiento y contactar con Seguridad Norte S.A.</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>{"presidente": "", "secretaria": "", "fecha": "", "lugar": "", "organizaciones": ["Limpiex S.L.", "Seguridad Norte S.A."]}</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr"/>
+      <c r="I39" t="inlineStr"/>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>json_schema</t>
+        </is>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>presidente,secretaria,fecha,lugar,organizaciones</t>
+        </is>
+      </c>
+      <c r="L39" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>LLM-NER-007</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>LLM_NER_EXTRACTION</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>NER_EXTRACTION</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>NER_EXTENDED</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>Extrae lugar y fecha.</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>Reunión extraordinaria en Sala de reuniones del edificio el 25 de febrero de 2026.</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>{"presidente": "", "secretaria": "", "fecha": "25/02/2026", "lugar": "Sala de reuniones del edificio", "organizaciones": []}</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr"/>
+      <c r="I40" t="inlineStr"/>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>json_schema</t>
+        </is>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>presidente,secretaria,fecha,lugar,organizaciones</t>
+        </is>
+      </c>
+      <c r="L40" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>LLM-NER-008</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>LLM_NER_EXTRACTION</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>NER_EXTRACTION</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>NER_EXTENDED</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Extrae cargos.</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>Manuel Ortega Medina asume la presidencia. Natalia Vázquez Gutiérrez actúa como secretaria.</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>{"presidente": "Manuel Ortega Medina", "secretaria": "Natalia Vázquez Gutiérrez", "fecha": "", "lugar": "", "organizaciones": []}</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr"/>
+      <c r="I41" t="inlineStr"/>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>json_schema</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>presidente,secretaria,fecha,lugar,organizaciones</t>
+        </is>
+      </c>
+      <c r="L41" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>LLM-NER-009</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>LLM_NER_EXTRACTION</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>NER_EXTRACTION</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>NER_EXTENDED</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>Extrae entidades de asistentes.</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>Asistentes: Beatriz Suárez Aguilar, Daniel Gutiérrez Moreno, Manuel Ortega Medina (Presidente).</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>{"presidente": "Manuel Ortega Medina", "secretaria": "", "fecha": "", "lugar": "", "organizaciones": []}</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr"/>
+      <c r="I42" t="inlineStr"/>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>json_schema</t>
+        </is>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>presidente,secretaria,fecha,lugar,organizaciones</t>
+        </is>
+      </c>
+      <c r="L42" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>LLM-NER-010</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>LLM_NER_EXTRACTION</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>NER_EXTRACTION</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>NER_EXTENDED</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>Extrae fecha y hora.</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>Acta de 25 de agosto de 2025. Inicio 19:30. Fin 21:00.</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>{"presidente": "", "secretaria": "", "fecha": "25/08/2025", "lugar": "Sala de reuniones del edificio", "organizaciones": []}</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr"/>
+      <c r="I43" t="inlineStr"/>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>json_schema</t>
+        </is>
+      </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>presidente,secretaria,fecha,lugar,organizaciones</t>
+        </is>
+      </c>
+      <c r="L43" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>LLM-NER-011</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>LLM_NER_EXTRACTION</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>NER_EXTRACTION</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>NER_EXTENDED</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>Extrae entidades de proveedor.</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>Se contrata Ascensores Vega S.L. para revisión del ascensor.</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>{"presidente": "", "secretaria": "", "fecha": "", "lugar": "", "organizaciones": ["Ascensores Vega S.L."]}</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr"/>
+      <c r="I44" t="inlineStr"/>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>json_schema</t>
+        </is>
+      </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>presidente,secretaria,fecha,lugar,organizaciones</t>
+        </is>
+      </c>
+      <c r="L44" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>LLM-NER-012</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>LLM_NER_EXTRACTION</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>NER_EXTRACTION</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>NER_EXTENDED</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>Extrae presidente y temas como organizaciones vacías.</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>Presidente: Jorge Moreno Navarro. Temas: calefacción, plagas.</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>{"presidente": "Jorge Moreno Navarro", "secretaria": "Natalia Vázquez Gutiérrez", "fecha": "25/02/2026", "lugar": "Sala de reuniones del edificio", "organizaciones": []}</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr"/>
+      <c r="I45" t="inlineStr"/>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>json_schema</t>
+        </is>
+      </c>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>presidente,secretaria,fecha,lugar,organizaciones</t>
+        </is>
+      </c>
+      <c r="L45" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>LLM-NER-013</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>LLM_NER_EXTRACTION</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>NER_EXTRACTION</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>NER_EXTENDED</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>Extrae entidades mínimas.</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>24 de febrero de 2025. Sala de reuniones del edificio.</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>{"presidente": "Juan Pérez Gutiérrez", "secretaria": "Rosa Aguilar Fernández", "fecha": "24/02/2025", "lugar": "Sala de reuniones del edificio", "organizaciones": []}</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr"/>
+      <c r="I46" t="inlineStr"/>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>json_schema</t>
+        </is>
+      </c>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>presidente,secretaria,fecha,lugar,organizaciones</t>
+        </is>
+      </c>
+      <c r="L46" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>LLM-NER-014</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>LLM_NER_EXTRACTION</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>NER_EXTRACTION</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>NER_EXTENDED</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>Extrae entidades de acta 2.</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>25/02/2025. Antonio Martínez López. Temas seguridad y estacionamiento.</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>{"presidente": "Antonio Martínez López", "secretaria": "Natalia Vázquez Gutiérrez", "fecha": "25/02/2025", "lugar": "Sala de reuniones del edificio", "organizaciones": []}</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr"/>
+      <c r="I47" t="inlineStr"/>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>json_schema</t>
+        </is>
+      </c>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>presidente,secretaria,fecha,lugar,organizaciones</t>
+        </is>
+      </c>
+      <c r="L47" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>LLM-NER-015</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>LLM_NER_EXTRACTION</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>NER_EXTRACTION</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>NER_EXTENDED</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>Extrae entidades con junta.</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>La Junta de Propietarios del edificio celebró sesión el 25/08/2026.</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>{"presidente": "Manuel Ortega Medina", "secretaria": "Natalia Vázquez Gutiérrez", "fecha": "25/08/2026", "lugar": "Sala de reuniones del edificio", "organizaciones": ["Junta de Propietarios"]}</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr"/>
+      <c r="I48" t="inlineStr"/>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>json_schema</t>
+        </is>
+      </c>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>presidente,secretaria,fecha,lugar,organizaciones</t>
+        </is>
+      </c>
+      <c r="L48" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>LLM-NER-016</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>LLM_NER_EXTRACTION</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>NER_EXTRACTION</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>NER_EXTENDED</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>Extrae entidades de cierre.</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>Se levanta la sesión a las 20:45. Presidente Manuel Ortega Medina. Secretaria Natalia Vázquez Gutiérrez.</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>{"presidente": "Manuel Ortega Medina", "secretaria": "Natalia Vázquez Gutiérrez", "fecha": "25/08/2026", "lugar": "Sala de reuniones del edificio", "organizaciones": []}</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr"/>
+      <c r="I49" t="inlineStr"/>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>json_schema</t>
+        </is>
+      </c>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>presidente,secretaria,fecha,lugar,organizaciones</t>
+        </is>
+      </c>
+      <c r="L49" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>LLM-MEM-001</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>LLM_MEMORY_CONDENSE</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>MEMORY_CONDENSE</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>MEMORY_BALANCED</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>Resume el hilo de conversación sobre el presidente.</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>Usuario: ¿Quién presidió? Asistente: Manuel Ortega Medina. Usuario: ¿Y la secretaria? Asistente: Natalia Vázquez Gutiérrez.
+Acta: Fecha 25/08/2026. Manuel Ortega Medina (Presidente), Natalia Vázquez Gutiérrez (Secretaria).</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>La reunión del 25/08/2026 fue presidida por Manuel Ortega Medina con Natalia Vázquez Gutiérrez como secretaria.</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>Manuel Ortega Medina,Natalia Vázquez Gutiérrez,25/08/2026,presidente,secretaria</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr"/>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>judge_qa,keyword_coverage</t>
+        </is>
+      </c>
+      <c r="K50" t="inlineStr"/>
+      <c r="L50" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>LLM-MEM-002</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>LLM_MEMORY_CONDENSE</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>MEMORY_CONDENSE</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>MEMORY_BALANCED</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>Condensa discusión sobre asistentes.</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>Usuario: ¿Cuántos vinieron? Asistente: 18 propietarios según ACTA 3.
+Acta: 25/08/2025, 18 propietarios, Beatriz Suárez Aguilar presidenta.</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>En el ACTA 3 del 25/08/2025 asistieron 18 propietarios; presidió Beatriz Suárez Aguilar.</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>18 propietarios,ACTA 3,Beatriz Suárez Aguilar</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr"/>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>judge_qa,keyword_coverage</t>
+        </is>
+      </c>
+      <c r="K51" t="inlineStr"/>
+      <c r="L51" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>LLM-MEM-003</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>LLM_MEMORY_CONDENSE</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>MEMORY_CONDENSE</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>MEMORY_BALANCED</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>Condensa tema ascensor.</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>Usuario: ascensor. Asistente: En ACTA 1 se acordó reparación. Usuario: ¿Y en ACTA 6? Asistente: También mantenimiento.
+Acta 6: Sistema eléctrico; ascensor; terrazas.</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>El ascensor se trató en ACTA 1 (reparación) y ACTA 6 (mantenimiento junto a sistema eléctrico y terrazas).</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>ascensor,reparación,mantenimiento,ACTA 1,ACTA 6</t>
+        </is>
+      </c>
+      <c r="I52" t="inlineStr"/>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>judge_qa,keyword_coverage</t>
+        </is>
+      </c>
+      <c r="K52" t="inlineStr"/>
+      <c r="L52" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>LLM-MEM-004</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>LLM_MEMORY_CONDENSE</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>MEMORY_CONDENSE</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>MEMORY_BALANCED</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>Condensa lugar y hora.</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>Usuario: ¿Dónde fue? Asistente: Sala del edificio. Usuario: ¿A qué hora? Asistente: 19:00 en ACTA 5.
+Acta 5: 25/02/2026, 19:00-20:30, Sala de reuniones del edificio.</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>ACTA 5 (25/02/2026): reunión en la sala del edificio de 19:00 a 20:30.</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>ACTA 5,19:00,Sala de reuniones,25/02/2026</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr"/>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>judge_qa,keyword_coverage</t>
+        </is>
+      </c>
+      <c r="K53" t="inlineStr"/>
+      <c r="L53" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>LLM-MEM-005</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>LLM_MEMORY_CONDENSE</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>MEMORY_CONDENSE</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>MEMORY_BALANCED</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>Condensa temas seguridad.</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>Usuario: cámaras. Asistente: ACTA 2 trata cámaras y estacionamiento. Usuario: ¿videovigilancia? Asistente: Sí en ACTA 6.
+Acta 2: cámaras, seguridad. Acta 6: videovigilancia.</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>Seguridad abordada en ACTA 2 (cámaras, estacionamiento) y ACTA 6 (videovigilancia).</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>cámaras,videovigilancia,seguridad,ACTA 2,ACTA 6</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr"/>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>judge_qa,keyword_coverage</t>
+        </is>
+      </c>
+      <c r="K54" t="inlineStr"/>
+      <c r="L54" t="inlineStr"/>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>LLM-MEM-006</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>LLM_MEMORY_CONDENSE</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>MEMORY_CONDENSE</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>MEMORY_BALANCED</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>Condensa presupuesto.</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>Usuario: presupuesto. Asistente: ACTA 1 incluye presupuesto anual.
+Acta 1: Estado de cuentas; presupuesto anual; reparación ascensor.</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>ACTA 1 trató estado de cuentas, presupuesto anual y reparación del ascensor.</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>presupuesto anual,estado de cuentas,ACTA 1</t>
+        </is>
+      </c>
+      <c r="I55" t="inlineStr"/>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>judge_qa,keyword_coverage</t>
+        </is>
+      </c>
+      <c r="K55" t="inlineStr"/>
+      <c r="L55" t="inlineStr"/>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>LLM-MEM-007</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>LLM_MEMORY_CONDENSE</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>MEMORY_CONDENSE</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>MEMORY_BALANCED</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>Condensa calefacción y plagas.</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>Usuario: temas ACTA 5. Asistente: calefacción y plagas.
+Acta 5: Calefacción; reglamento; plagas; salidas emergencia.</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>ACTA 5 cubrió calefacción, reglamento de convivencia, plagas y salidas de emergencia.</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>calefacción,plagas,ACTA 5,salidas de emergencia</t>
+        </is>
+      </c>
+      <c r="I56" t="inlineStr"/>
+      <c r="J56" t="inlineStr">
+        <is>
+          <t>judge_qa,keyword_coverage</t>
+        </is>
+      </c>
+      <c r="K56" t="inlineStr"/>
+      <c r="L56" t="inlineStr"/>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>LLM-MEM-008</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>LLM_MEMORY_CONDENSE</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>MEMORY_CONDENSE</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>MEMORY_BALANCED</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>Condensa piscina y jardines.</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>Usuario: zonas comunes. Asistente: piscina y jardines en ACTA 3.
+Acta 3: piscina, jardines, bicicletas.</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>ACTA 3 abordó piscina, jardines y almacenamiento de bicicletas.</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>piscina,jardines,bicicletas,ACTA 3</t>
+        </is>
+      </c>
+      <c r="I57" t="inlineStr"/>
+      <c r="J57" t="inlineStr">
+        <is>
+          <t>judge_qa,keyword_coverage</t>
+        </is>
+      </c>
+      <c r="K57" t="inlineStr"/>
+      <c r="L57" t="inlineStr"/>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>LLM-MEM-009</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>LLM_MEMORY_CONDENSE</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>MEMORY_CONDENSE</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>MEMORY_BALANCED</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>Condensa secretaria histórica.</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>Usuario: secretarias. Asistente: Rosa en ACTA 1, Natalia en varias actas.
+Acta 1: Rosa Aguilar Fernández. Acta 6: Natalia Vázquez Gutiérrez.</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>Rosa Aguilar Fernández secretaria en ACTA 1; Natalia Vázquez Gutiérrez en ACTA 6 y otras actas.</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>Rosa Aguilar Fernández,Natalia Vázquez Gutiérrez,secretaria</t>
+        </is>
+      </c>
+      <c r="I58" t="inlineStr"/>
+      <c r="J58" t="inlineStr">
+        <is>
+          <t>judge_qa,keyword_coverage</t>
+        </is>
+      </c>
+      <c r="K58" t="inlineStr"/>
+      <c r="L58" t="inlineStr"/>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>LLM-MEM-010</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>LLM_MEMORY_CONDENSE</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>MEMORY_CONDENSE</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>MEMORY_BALANCED</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>Condensa decisión portal.</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>Usuario: portal. Asistente: pintura ACTA 1, renovación ACTA 3.
+Acta 1: pintura portal. Acta 3: renovación portal.</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>Mejoras del portal: pintura (ACTA 1) y renovación (ACTA 3).</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>portal,pintura,renovación,ACTA 1,ACTA 3</t>
+        </is>
+      </c>
+      <c r="I59" t="inlineStr"/>
+      <c r="J59" t="inlineStr">
+        <is>
+          <t>judge_qa,keyword_coverage</t>
+        </is>
+      </c>
+      <c r="K59" t="inlineStr"/>
+      <c r="L59" t="inlineStr"/>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>LLM-MEM-011</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>LLM_MEMORY_CONDENSE</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>MEMORY_CONDENSE</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>MEMORY_BALANCED</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>Condensa horarios múltiples actas.</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>Usuario: horarios. Asistente: ACTA 1 19:00-20:30, ACTA 3 19:30-21:00.
+Actas con horarios indicados.</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>Horarios típicos: ACTA 1 (19:00-20:30) y ACTA 3 (19:30-21:00) en sala del edificio.</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>19:00,19:30,ACTA 1,ACTA 3</t>
+        </is>
+      </c>
+      <c r="I60" t="inlineStr"/>
+      <c r="J60" t="inlineStr">
+        <is>
+          <t>judge_qa,keyword_coverage</t>
+        </is>
+      </c>
+      <c r="K60" t="inlineStr"/>
+      <c r="L60" t="inlineStr"/>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>LLM-MEM-012</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>LLM_MEMORY_CONDENSE</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>MEMORY_CONDENSE</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>MEMORY_BALANCED</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>Condensa iluminación.</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>Usuario: iluminación. Asistente: ACTA 3 y ACTA 5.
+Acta 3: iluminación. Acta 5: iluminación.</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>Iluminación tratada en ACTA 3 y ACTA 5.</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>iluminación,ACTA 3,ACTA 5</t>
+        </is>
+      </c>
+      <c r="I61" t="inlineStr"/>
+      <c r="J61" t="inlineStr">
+        <is>
+          <t>judge_qa,keyword_coverage</t>
+        </is>
+      </c>
+      <c r="K61" t="inlineStr"/>
+      <c r="L61" t="inlineStr"/>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>LLM-MEM-013</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>LLM_MEMORY_CONDENSE</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>MEMORY_CONDENSE</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>MEMORY_BALANCED</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>Condensa abstención previa.</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>Usuario: multa ruido. Asistente: no consta. Usuario: ok resume.
+Acta sin mención de multas por ruido.</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>No hay información sobre multas por ruido en las actas consultadas.</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>no consta,multa,ruido</t>
+        </is>
+      </c>
+      <c r="I62" t="inlineStr"/>
+      <c r="J62" t="inlineStr">
+        <is>
+          <t>judge_qa,keyword_coverage</t>
+        </is>
+      </c>
+      <c r="K62" t="inlineStr"/>
+      <c r="L62" t="inlineStr"/>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>LLM-MEM-014</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>LLM_MEMORY_CONDENSE</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>MEMORY_CONDENSE</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>MEMORY_BALANCED</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>Condensa sistema eléctrico.</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>Usuario: electricidad. Asistente: ACTA 6 sistema eléctrico.
+Acta 6: Sistema eléctrico; ascensor; terrazas; videovigilancia.</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>ACTA 6 trató sistema eléctrico, ascensor, terrazas y videovigilancia.</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>sistema eléctrico,ACTA 6,ascensor</t>
+        </is>
+      </c>
+      <c r="I63" t="inlineStr"/>
+      <c r="J63" t="inlineStr">
+        <is>
+          <t>judge_qa,keyword_coverage</t>
+        </is>
+      </c>
+      <c r="K63" t="inlineStr"/>
+      <c r="L63" t="inlineStr"/>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>LLM-MEM-015</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>LLM_MEMORY_CONDENSE</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>MEMORY_CONDENSE</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>MEMORY_BALANCED</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>Condensa normas convivencia.</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>Usuario: convivencia. Asistente: ACTA 1 y ACTA 5.
+Acta 1: normas convivencia. Acta 5: reglamento convivencia.</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>Normas o reglamento de convivencia discutidos en ACTA 1 y ACTA 5.</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>convivencia,reglamento,ACTA 1,ACTA 5</t>
+        </is>
+      </c>
+      <c r="I64" t="inlineStr"/>
+      <c r="J64" t="inlineStr">
+        <is>
+          <t>judge_qa,keyword_coverage</t>
+        </is>
+      </c>
+      <c r="K64" t="inlineStr"/>
+      <c r="L64" t="inlineStr"/>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>LLM-MEM-016</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>LLM_MEMORY_CONDENSE</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>MEMORY_CONDENSE</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>MEMORY_BALANCED</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>Condensa resumen sesión completa.</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>Usuario: resume ACTA 6. Asistente: presidente Manuel, 19 asistentes, temas eléctrico y ascensor.
+Acta 6 completa: 25/08/2026, Manuel Ortega Medina, 19 asistentes, sistema eléctrico, ascensor, terrazas, videovigilancia.</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>ACTA 6 (25/08/2026): Manuel Ortega Medina preside con 19 asistentes; temas sistema eléctrico, ascensor, terrazas y videovigilancia.</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>ACTA 6,Manuel Ortega Medina,19 asistentes,sistema eléctrico,ascensor</t>
+        </is>
+      </c>
+      <c r="I65" t="inlineStr"/>
+      <c r="J65" t="inlineStr">
+        <is>
+          <t>judge_qa,keyword_coverage</t>
+        </is>
+      </c>
+      <c r="K65" t="inlineStr"/>
+      <c r="L65" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>